<commit_message>
Deploy Atlas site from f920a73fec6d424a52740d9d75619c9e40ddd3e0
</commit_message>
<xml_diff>
--- a/downloads/roles/roles-responsibilities-authority-workbook.xlsx
+++ b/downloads/roles/roles-responsibilities-authority-workbook.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Start Here'!$A$2:$B$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Role Registry'!$A$2:$H$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Process Role Map'!$A$2:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Artifact Ownership'!$A$2:$K$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Artifact Ownership'!$A$2:$K$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lifecycle Handoffs'!$A$2:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decision Authority'!$A$2:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Assignment Workshop'!$A$2:$J$4</definedName>
@@ -4173,7 +4173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4694,27 +4694,27 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ART-RSK-001</t>
+          <t>ART-STK-003</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Risk Register</t>
+          <t>Stakeholder Engagement Assessment Matrix</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Risk Owner; Issue or Impediment Owner; Delivery Team</t>
+          <t>Project Manager; Project Team Member</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Risk Owner; Project Manager</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Subject-Matter Expert; Stakeholder</t>
+          <t>Project Team Member; Stakeholder; Sponsor; Product Owner</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Compliance Authority</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -4735,22 +4735,22 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>ART-INT-001</t>
+          <t>ART-RSK-001</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Assumption Log</t>
+          <t>Risk Register</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Project Team Member</t>
+          <t>Project Manager; Risk Owner; Issue or Impediment Owner; Delivery Team</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Knowledge or Records Custodian</t>
+          <t>Risk Owner; Project Manager</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Project Manager; Compliance Authority</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -4776,22 +4776,22 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>ART-CHR-001</t>
+          <t>ART-INT-001</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Project Charter</t>
+          <t>Assumption Log</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Project Manager</t>
+          <t>Project Manager; Project Team Member</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Benefit Owner</t>
+          <t>Project Manager; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -4809,11 +4809,7 @@
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
+      <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr"/>
@@ -4821,27 +4817,27 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>ART-SCP-002</t>
+          <t>ART-CHR-001</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Project Scope Statement</t>
+          <t>Project Charter</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Business Analyst; Project Manager</t>
+          <t>Sponsor; Project Manager</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Knowledge or Records Custodian</t>
+          <t>Sponsor; Benefit Owner</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Customer or Acceptance Authority; Product Owner; Stakeholder; Delivery Team</t>
+          <t>Subject-Matter Expert; Stakeholder</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -4851,10 +4847,14 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Customer or Acceptance Authority; Product Owner</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
       <c r="I16" s="3" t="inlineStr"/>
       <c r="J16" s="3" t="inlineStr"/>
       <c r="K16" s="3" t="inlineStr"/>
@@ -4862,17 +4862,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>ART-INT-002</t>
+          <t>ART-SCP-002</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Lessons Learned Register</t>
+          <t>Project Scope Statement</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Project Team Member</t>
+          <t>Business Analyst; Project Manager</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Subject-Matter Expert; Stakeholder</t>
+          <t>Customer or Acceptance Authority; Product Owner; Stakeholder; Delivery Team</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Customer or Acceptance Authority; Product Owner</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -4903,12 +4903,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>ART-DEL-001</t>
+          <t>ART-INT-002</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Deliverables</t>
+          <t>Lessons Learned Register</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -4944,17 +4944,17 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ART-CHG-001</t>
+          <t>ART-DEL-001</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Change Requests</t>
+          <t>Deliverables</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Stakeholder; Project Manager; Delivery Team</t>
+          <t>Project Manager; Project Team Member</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -4974,14 +4974,10 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Change Authority or CCB</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Change Authority or CCB</t>
-        </is>
-      </c>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr"/>
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr"/>
@@ -4989,17 +4985,17 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ART-SCH-004</t>
+          <t>ART-CHG-001</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Project Schedule</t>
+          <t>Change Requests</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Project Team Member</t>
+          <t>Stakeholder; Project Manager; Delivery Team</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -5019,10 +5015,14 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr"/>
+          <t>Project Manager; Change Authority or CCB</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Change Authority or CCB</t>
+        </is>
+      </c>
       <c r="I20" s="3" t="inlineStr"/>
       <c r="J20" s="3" t="inlineStr"/>
       <c r="K20" s="3" t="inlineStr"/>
@@ -5030,12 +5030,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>ART-SCH-005</t>
+          <t>ART-SCH-004</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Schedule Baseline</t>
+          <t>Project Schedule</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -5071,12 +5071,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>ART-CST-001</t>
+          <t>ART-SCH-005</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Cost Estimates</t>
+          <t>Schedule Baseline</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -5112,12 +5112,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>ART-CST-002</t>
+          <t>ART-CST-001</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Cost Baseline</t>
+          <t>Cost Estimates</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -5153,27 +5153,27 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>ART-PRC-003</t>
+          <t>ART-CST-002</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Agreements</t>
+          <t>Cost Baseline</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Procurement or Contract Authority; Project Manager</t>
+          <t>Project Manager; Project Team Member</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Procurement or Contract Authority; Knowledge or Records Custodian</t>
+          <t>Project Manager; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Seller or Supplier; Subject-Matter Expert; Compliance Authority</t>
+          <t>Subject-Matter Expert; Stakeholder</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -5183,14 +5183,10 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Procurement or Contract Authority</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Procurement or Contract Authority</t>
-        </is>
-      </c>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr"/>
       <c r="J24" s="3" t="inlineStr"/>
       <c r="K24" s="3" t="inlineStr"/>
@@ -5198,27 +5194,27 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>ART-WPI-001</t>
+          <t>ART-PRC-003</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Work Performance Information</t>
+          <t>Agreements</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Project Team Member</t>
+          <t>Procurement or Contract Authority; Project Manager</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Knowledge or Records Custodian</t>
+          <t>Procurement or Contract Authority; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Subject-Matter Expert; Stakeholder</t>
+          <t>Seller or Supplier; Subject-Matter Expert; Compliance Authority</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -5228,10 +5224,14 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+          <t>Procurement or Contract Authority</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Procurement or Contract Authority</t>
+        </is>
+      </c>
       <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr"/>
       <c r="K25" s="3" t="inlineStr"/>
@@ -5239,12 +5239,12 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>ART-WPR-001</t>
+          <t>ART-WPI-001</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Work Performance Reports</t>
+          <t>Work Performance Information</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -5280,22 +5280,22 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>ART-BIZ-001</t>
+          <t>ART-WPR-001</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Business Case</t>
+          <t>Work Performance Reports</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Project Manager</t>
+          <t>Project Manager; Project Team Member</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Benefit Owner</t>
+          <t>Project Manager; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -5313,11 +5313,7 @@
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
+      <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr"/>
       <c r="K27" s="3" t="inlineStr"/>
@@ -5325,12 +5321,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>ART-BEN-001</t>
+          <t>ART-BIZ-001</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Benefits Management Information</t>
+          <t>Business Case</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -5370,22 +5366,22 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>ART-RSK-003</t>
+          <t>ART-BEN-001</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Risk Report</t>
+          <t>Benefits Management Information</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Risk Owner; Issue or Impediment Owner; Delivery Team</t>
+          <t>Sponsor; Project Manager</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Risk Owner; Project Manager</t>
+          <t>Sponsor; Benefit Owner</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -5400,10 +5396,14 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Compliance Authority</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr"/>
       <c r="K29" s="3" t="inlineStr"/>
@@ -5411,12 +5411,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>ART-ISS-001</t>
+          <t>ART-RSK-003</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Issue Log</t>
+          <t>Risk Report</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Issue or Impediment Owner; Project Manager</t>
+          <t>Risk Owner; Project Manager</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -5452,12 +5452,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>ART-ISS-002</t>
+          <t>ART-ISS-001</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Impediment Record</t>
+          <t>Issue Log</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -5493,22 +5493,22 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>ART-CHG-004</t>
+          <t>ART-ISS-002</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Change Log</t>
+          <t>Impediment Record</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Stakeholder; Project Manager; Delivery Team</t>
+          <t>Project Manager; Risk Owner; Issue or Impediment Owner; Delivery Team</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Knowledge or Records Custodian</t>
+          <t>Issue or Impediment Owner; Project Manager</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Change Authority or CCB</t>
+          <t>Project Manager; Compliance Authority</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
@@ -5534,22 +5534,22 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>ART-QLT-006</t>
+          <t>ART-CHG-004</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Quality Reports</t>
+          <t>Change Log</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Quality Authority; Delivery Team</t>
+          <t>Stakeholder; Project Manager; Delivery Team</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Quality Authority; Knowledge or Records Custodian</t>
+          <t>Project Manager; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -5564,27 +5564,23 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Quality Authority</t>
+          <t>Project Manager; Change Authority or CCB</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>Quality Authority</t>
-        </is>
-      </c>
+      <c r="I33" s="3" t="inlineStr"/>
       <c r="J33" s="3" t="inlineStr"/>
       <c r="K33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>ART-QLT-007</t>
+          <t>ART-QLT-006</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Test and Evaluation Documents</t>
+          <t>Quality Reports</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -5624,22 +5620,22 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>ART-CMP-001</t>
+          <t>ART-QLT-007</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Compliance Evidence and Traceability</t>
+          <t>Test and Evaluation Documents</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Compliance Authority; Quality Authority</t>
+          <t>Quality Authority; Delivery Team</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Compliance Authority; Knowledge or Records Custodian</t>
+          <t>Quality Authority; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -5654,13 +5650,13 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Compliance Authority</t>
+          <t>Quality Authority</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Compliance Authority</t>
+          <t>Quality Authority</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr"/>
@@ -5669,27 +5665,27 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>ART-PRC-004</t>
+          <t>ART-CMP-001</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Procurement Strategy</t>
+          <t>Compliance Evidence and Traceability</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Procurement or Contract Authority; Project Manager</t>
+          <t>Compliance Authority; Quality Authority</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Procurement or Contract Authority; Knowledge or Records Custodian</t>
+          <t>Compliance Authority; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Seller or Supplier; Subject-Matter Expert; Compliance Authority</t>
+          <t>Subject-Matter Expert; Stakeholder</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -5699,27 +5695,27 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Procurement or Contract Authority</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Procurement or Contract Authority</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr"/>
+          <t>Compliance Authority</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Compliance Authority</t>
+        </is>
+      </c>
       <c r="J36" s="3" t="inlineStr"/>
       <c r="K36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>ART-PRC-005</t>
+          <t>ART-PRC-004</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Procurement Statement of Work</t>
+          <t>Procurement Strategy</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -5759,12 +5755,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>ART-PRC-006</t>
+          <t>ART-PRC-005</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Source-Selection Criteria</t>
+          <t>Procurement Statement of Work</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -5804,12 +5800,12 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>ART-PRC-007</t>
+          <t>ART-PRC-006</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Closed Procurement</t>
+          <t>Source-Selection Criteria</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -5849,27 +5845,27 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>ART-TRN-001</t>
+          <t>ART-PRC-007</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Transition Package</t>
+          <t>Closed Procurement</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Project Team Member</t>
+          <t>Procurement or Contract Authority; Project Manager</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Project Manager; Knowledge or Records Custodian</t>
+          <t>Procurement or Contract Authority; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Operations or Service Owner; Delivery Team; Quality Authority; Compliance Authority</t>
+          <t>Seller or Supplier; Subject-Matter Expert; Compliance Authority</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -5879,31 +5875,27 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Procurement or Contract Authority</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>Operations or Service Owner</t>
+          <t>Procurement or Contract Authority</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr"/>
       <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr">
-        <is>
-          <t>Operations or Service Owner</t>
-        </is>
-      </c>
+      <c r="K40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>ART-CLS-001</t>
+          <t>ART-TRN-001</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Final Report</t>
+          <t>Transition Package</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -5918,7 +5910,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Customer or Acceptance Authority; Operations or Service Owner; Benefit Owner; Procurement or Contract Authority</t>
+          <t>Operations or Service Owner; Delivery Team; Quality Authority; Compliance Authority</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -5933,26 +5925,26 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Operations or Service Owner</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr"/>
       <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Knowledge or Records Custodian; Operations or Service Owner</t>
+          <t>Operations or Service Owner</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>ART-CLS-002</t>
+          <t>ART-CLS-001</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Formal Closure Record</t>
+          <t>Final Report</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -5996,27 +5988,27 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>ART-BEN-002</t>
+          <t>ART-CLS-002</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Benefits Handoff Record</t>
+          <t>Formal Closure Record</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Project Manager</t>
+          <t>Project Manager; Project Team Member</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Benefit Owner</t>
+          <t>Project Manager; Knowledge or Records Custodian</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Subject-Matter Expert; Stakeholder</t>
+          <t>Customer or Acceptance Authority; Operations or Service Owner; Benefit Owner; Procurement or Contract Authority</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -6031,19 +6023,68 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Sponsor; Benefit Owner</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr"/>
       <c r="K43" s="3" t="inlineStr">
         <is>
+          <t>Knowledge or Records Custodian; Operations or Service Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>ART-BEN-002</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Benefits Handoff Record</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor; Project Manager</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor; Benefit Owner</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Subject-Matter Expert; Stakeholder</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Project Manager; Project Team Member</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor; Benefit Owner</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr"/>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
           <t>Benefit Owner</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K43"/>
+  <autoFilter ref="A2:K44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Deploy Atlas site from 7d0ae773d2ea8e0be28758ef4ea6a9a41e8ebdfd
</commit_message>
<xml_diff>
--- a/downloads/roles/roles-responsibilities-authority-workbook.xlsx
+++ b/downloads/roles/roles-responsibilities-authority-workbook.xlsx
@@ -761,7 +761,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Provides governance support, standards, assurance, and portfolio-level coordination.</t>
+          <t>Provides contextual governance, tailoring, coaching, assurance, knowledge, tooling, measurement, and portfolio-level coordination where the organization delegates those functions.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Is not automatically the project sponsor or project manager.</t>
+          <t>Is not automatically the project sponsor or project manager and does not control every team decision merely because delivery is adaptive.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">

</xml_diff>